<commit_message>
feat: complete initial cloud integration
</commit_message>
<xml_diff>
--- a/outputs/019fc5c9/业务进度管理微信小程序开发排期.xlsx
+++ b/outputs/019fc5c9/业务进度管理微信小程序开发排期.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总体计划" sheetId="1" r:id="Rdf03c720480244b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务排期" sheetId="2" r:id="Rb66498cad3164581"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="里程碑与验收" sheetId="3" r:id="R1c12a5adccf04c64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总体计划" sheetId="1" r:id="R5cd9d3954c364707"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务排期" sheetId="2" r:id="Raacfac5ea44844af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="里程碑与验收" sheetId="3" r:id="R8c7601bd4ef3479f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -622,7 +622,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="项目组" id="{C954A3D2-454B-436F-AE3B-24CE5D5DF107}"/>
+  <xltc:person displayName="项目组" id="{CA5F781C-136C-4ABE-A208-55308657896E}"/>
 </xltc:personList>
 </file>
 
@@ -1696,7 +1696,7 @@
         <x:v>OpenID 唯一建档且状态可控</x:v>
       </x:c>
       <x:c r="K10" s="98" t="str">
-        <x:v>未开始</x:v>
+        <x:v>进行中</x:v>
       </x:c>
       <x:c r="L10" s="127" t="str">
         <x:v>P0</x:v>
@@ -1735,7 +1735,7 @@
         <x:v>可创建含至少一个节点的业务线</x:v>
       </x:c>
       <x:c r="K11" s="98" t="str">
-        <x:v>未开始</x:v>
+        <x:v>进行中</x:v>
       </x:c>
       <x:c r="L11" s="127" t="str">
         <x:v>P0</x:v>
@@ -1774,7 +1774,7 @@
         <x:v>成员只能看到关联业务</x:v>
       </x:c>
       <x:c r="K12" s="98" t="str">
-        <x:v>未开始</x:v>
+        <x:v>进行中</x:v>
       </x:c>
       <x:c r="L12" s="127" t="str">
         <x:v>P0</x:v>
@@ -1813,7 +1813,7 @@
         <x:v>并发更新不覆盖他人改动</x:v>
       </x:c>
       <x:c r="K13" s="98" t="str">
-        <x:v>未开始</x:v>
+        <x:v>进行中</x:v>
       </x:c>
       <x:c r="L13" s="127" t="str">
         <x:v>P0</x:v>
@@ -1852,7 +1852,7 @@
         <x:v>非管理员请求被拒绝并留痕</x:v>
       </x:c>
       <x:c r="K14" s="98" t="str">
-        <x:v>未开始</x:v>
+        <x:v>进行中</x:v>
       </x:c>
       <x:c r="L14" s="127" t="str">
         <x:v>P0</x:v>
@@ -2593,7 +2593,7 @@
         <x:v>核心权限和状态机覆盖率达标</x:v>
       </x:c>
       <x:c r="K33" s="98" t="str">
-        <x:v>未开始</x:v>
+        <x:v>进行中</x:v>
       </x:c>
       <x:c r="L33" s="127" t="str">
         <x:v>P0</x:v>

</xml_diff>